<commit_message>
Refaz a Carteira Sugerida no formato de proposta e adiciona Planejamento + Tabela Periódica
- Carteira Sugerida vira uma proposta no estilo modelo de carteira:
  cabeçalho com banner de Patrimônio Proposto, tabela com Classe,
  Ativo, Carência (dias) e Liquidez (dias), pizza de composição por
  classe, barras de distribuição de liquidez, blocos de Otimizações e
  Racional por movimentação; o comparativo Atual x Sugerida continua
  ao final.
- Planejamento: premissas (idade, patrimônio, aplicação mensal,
  inflação, CDI, IR, %CDI esperado, renda desejada, INSS, taxa real),
  cálculo de patrimônio necessário e parcela mensal nos cenários
  Viver de Renda e Consumo com Sucessão, objetivos de vida 1-6 anos
  e gráfico de Projeção Patrimonial em R$ de hoje.
- Tabela Periódica: grade de retornos anuais por índice/classe com
  cálculo automático do acumulado e color-scale por ano (melhor verde,
  pior vermelho).

https://claude.ai/code/session_012B6pvzwHHmCv3nAgYhFWdt
</commit_message>
<xml_diff>
--- a/gestao_carteiras.xlsx
+++ b/gestao_carteiras.xlsx
@@ -11,7 +11,9 @@
     <sheet name="Aplicacoes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Carteira do Cliente" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Carteira Sugerida" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Planejamento" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tabela Periódica" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Instruções" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,12 +22,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="165" formatCode="R$ #,##0.00;[Red]-R$ #,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0.0000%"/>
+    <numFmt numFmtId="168" formatCode="0.00%;[Red]-0.00%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +71,32 @@
       <sz val="10"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
       <i val="1"/>
       <color rgb="005B6470"/>
       <sz val="9"/>
@@ -81,7 +111,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -118,6 +148,11 @@
         <fgColor rgb="00F0F2F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C0392B"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -145,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -250,10 +285,19 @@
     <xf numFmtId="1" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -263,13 +307,61 @@
     <xf numFmtId="166" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -448,7 +540,62 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Alocação atual x sugerida (%)</a:t>
+              <a:t>Composição por Classe de Ativos</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Carteira Sugerida'!$Q$8:$Q$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Carteira Sugerida'!$R$8:$R$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showPercent val="1"/>
+        </dLbls>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Distribuição de Liquidez (R$ por D+)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -461,11 +608,6 @@
         <ser>
           <idx val="0"/>
           <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Carteira Sugerida'!B37</f>
-            </strRef>
-          </tx>
           <spPr>
             <a:ln>
               <a:prstDash val="solid"/>
@@ -473,36 +615,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Carteira Sugerida'!$A$38:$A$45</f>
+              <f>'Carteira Sugerida'!$S$8:$S$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Carteira Sugerida'!$B$38:$B$45</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Carteira Sugerida'!C37</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Carteira Sugerida'!$A$38:$A$45</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Carteira Sugerida'!$C$38:$C$45</f>
+              <f>'Carteira Sugerida'!$T$8:$T$18</f>
             </numRef>
           </val>
         </ser>
@@ -517,6 +635,21 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Liquidez (dias)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -530,7 +663,149 @@
         <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
-        <numFmt formatCode="0%" sourceLinked="0"/>
+        <numFmt formatCode="R$ #,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Projeção Patrimonial — Independência Financeira &amp; Aposentadoria</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <areaChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Planejamento'!I34</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Planejamento'!$H$35:$H$74</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Planejamento'!$I$35:$I$74</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </areaChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Planejamento'!J34</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Planejamento'!$J$35:$J$74</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Idade</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Patrimônio (R$)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="R$ #,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -539,7 +814,7 @@
     <legend>
       <legendPos val="r"/>
     </legend>
-    <plotVisOnly val="1"/>
+    <plotVisOnly val="0"/>
     <dispBlanksAs val="gap"/>
   </chart>
 </chartSpace>
@@ -576,12 +851,61 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3420000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3420000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>47</row>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6120000" cy="3240000"/>
+    <ext cx="7920000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -28974,26 +29298,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:T67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="2" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CARTEIRA SUGERIDA</t>
+          <t>PROPOSTA DE CARTEIRA</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="22" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Cliente:</t>
@@ -29003,36 +29338,35 @@
         <f>'Carteira do Cliente'!B3</f>
         <v/>
       </c>
-      <c r="E3" s="37" t="inlineStr">
+      <c r="H3" s="37" t="inlineStr">
         <is>
-          <t>Selecione o cliente na aba 'Carteira do Cliente'.</t>
+          <t>PATRIMÔNIO PROPOSTO</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="17" t="inlineStr">
         <is>
-          <t>Patrimônio atual:</t>
+          <t>Patrimônio Atual:</t>
         </is>
       </c>
       <c r="B4" s="20">
         <f>'Carteira do Cliente'!B6</f>
+        <v/>
+      </c>
+      <c r="H4" s="38">
+        <f>SUM(E8:E32)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="22" t="inlineStr">
         <is>
-          <t>CARTEIRA ATUAL POR CLASSE</t>
+          <t>CARTEIRA RECOMENDADA</t>
         </is>
       </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>CARTEIRA SUGERIDA — PREENCHA</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+    </row>
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Classe</t>
@@ -29040,596 +29374,908 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Saldo Atual (R$)</t>
+          <t>Ativo sugerido</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Carência
+(dias corridos)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Liquidez
+(D + dias)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Valor (R$)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="Q7" s="39" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="R7" s="39" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="S7" s="39" t="inlineStr">
+        <is>
+          <t>D+</t>
+        </is>
+      </c>
+      <c r="T7" s="39" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="n"/>
+      <c r="B8" s="23" t="n"/>
+      <c r="C8" s="40" t="n"/>
+      <c r="D8" s="40" t="n"/>
+      <c r="E8" s="41" t="n"/>
+      <c r="F8" s="25">
+        <f>IFERROR($E8/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+      <c r="Q8">
+        <f>'Carteira do Cliente'!A11</f>
+        <v/>
+      </c>
+      <c r="R8">
+        <f>IF($Q8="",0,SUMIFS($E$8:$E$32,$A$8:$A$32,$Q8))</f>
+        <v/>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <f>SUMIFS($E$8:$E$32,$D$8:$D$32,$S8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="n"/>
+      <c r="B9" s="23" t="n"/>
+      <c r="C9" s="40" t="n"/>
+      <c r="D9" s="40" t="n"/>
+      <c r="E9" s="41" t="n"/>
+      <c r="F9" s="25">
+        <f>IFERROR($E9/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+      <c r="Q9">
+        <f>'Carteira do Cliente'!A12</f>
+        <v/>
+      </c>
+      <c r="R9">
+        <f>IF($Q9="",0,SUMIFS($E$8:$E$32,$A$8:$A$32,$Q9))</f>
+        <v/>
+      </c>
+      <c r="S9" t="n">
+        <v>1</v>
+      </c>
+      <c r="T9">
+        <f>SUMIFS($E$8:$E$32,$D$8:$D$32,$S9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="n"/>
+      <c r="B10" s="23" t="n"/>
+      <c r="C10" s="40" t="n"/>
+      <c r="D10" s="40" t="n"/>
+      <c r="E10" s="41" t="n"/>
+      <c r="F10" s="25">
+        <f>IFERROR($E10/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+      <c r="Q10">
+        <f>'Carteira do Cliente'!A13</f>
+        <v/>
+      </c>
+      <c r="R10">
+        <f>IF($Q10="",0,SUMIFS($E$8:$E$32,$A$8:$A$32,$Q10))</f>
+        <v/>
+      </c>
+      <c r="S10" t="n">
+        <v>10</v>
+      </c>
+      <c r="T10">
+        <f>SUMIFS($E$8:$E$32,$D$8:$D$32,$S10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="n"/>
+      <c r="B11" s="23" t="n"/>
+      <c r="C11" s="40" t="n"/>
+      <c r="D11" s="40" t="n"/>
+      <c r="E11" s="41" t="n"/>
+      <c r="F11" s="25">
+        <f>IFERROR($E11/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+      <c r="Q11">
+        <f>'Carteira do Cliente'!A14</f>
+        <v/>
+      </c>
+      <c r="R11">
+        <f>IF($Q11="",0,SUMIFS($E$8:$E$32,$A$8:$A$32,$Q11))</f>
+        <v/>
+      </c>
+      <c r="S11" t="n">
+        <v>30</v>
+      </c>
+      <c r="T11">
+        <f>SUMIFS($E$8:$E$32,$D$8:$D$32,$S11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="n"/>
+      <c r="B12" s="23" t="n"/>
+      <c r="C12" s="40" t="n"/>
+      <c r="D12" s="40" t="n"/>
+      <c r="E12" s="41" t="n"/>
+      <c r="F12" s="25">
+        <f>IFERROR($E12/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+      <c r="Q12">
+        <f>'Carteira do Cliente'!A15</f>
+        <v/>
+      </c>
+      <c r="R12">
+        <f>IF($Q12="",0,SUMIFS($E$8:$E$32,$A$8:$A$32,$Q12))</f>
+        <v/>
+      </c>
+      <c r="S12" t="n">
+        <v>45</v>
+      </c>
+      <c r="T12">
+        <f>SUMIFS($E$8:$E$32,$D$8:$D$32,$S12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="n"/>
+      <c r="B13" s="23" t="n"/>
+      <c r="C13" s="40" t="n"/>
+      <c r="D13" s="40" t="n"/>
+      <c r="E13" s="41" t="n"/>
+      <c r="F13" s="25">
+        <f>IFERROR($E13/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+      <c r="Q13">
+        <f>'Carteira do Cliente'!A16</f>
+        <v/>
+      </c>
+      <c r="R13">
+        <f>IF($Q13="",0,SUMIFS($E$8:$E$32,$A$8:$A$32,$Q13))</f>
+        <v/>
+      </c>
+      <c r="S13" t="n">
+        <v>90</v>
+      </c>
+      <c r="T13">
+        <f>SUMIFS($E$8:$E$32,$D$8:$D$32,$S13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="23" t="n"/>
+      <c r="C14" s="40" t="n"/>
+      <c r="D14" s="40" t="n"/>
+      <c r="E14" s="41" t="n"/>
+      <c r="F14" s="25">
+        <f>IFERROR($E14/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+      <c r="Q14">
+        <f>'Carteira do Cliente'!A17</f>
+        <v/>
+      </c>
+      <c r="R14">
+        <f>IF($Q14="",0,SUMIFS($E$8:$E$32,$A$8:$A$32,$Q14))</f>
+        <v/>
+      </c>
+      <c r="S14" t="n">
+        <v>180</v>
+      </c>
+      <c r="T14">
+        <f>SUMIFS($E$8:$E$32,$D$8:$D$32,$S14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="n"/>
+      <c r="B15" s="23" t="n"/>
+      <c r="C15" s="40" t="n"/>
+      <c r="D15" s="40" t="n"/>
+      <c r="E15" s="41" t="n"/>
+      <c r="F15" s="25">
+        <f>IFERROR($E15/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+      <c r="Q15">
+        <f>'Carteira do Cliente'!A18</f>
+        <v/>
+      </c>
+      <c r="R15">
+        <f>IF($Q15="",0,SUMIFS($E$8:$E$32,$A$8:$A$32,$Q15))</f>
+        <v/>
+      </c>
+      <c r="S15" t="n">
+        <v>270</v>
+      </c>
+      <c r="T15">
+        <f>SUMIFS($E$8:$E$32,$D$8:$D$32,$S15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="n"/>
+      <c r="B16" s="23" t="n"/>
+      <c r="C16" s="40" t="n"/>
+      <c r="D16" s="40" t="n"/>
+      <c r="E16" s="41" t="n"/>
+      <c r="F16" s="25">
+        <f>IFERROR($E16/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+      <c r="S16" t="n">
+        <v>365</v>
+      </c>
+      <c r="T16">
+        <f>SUMIFS($E$8:$E$32,$D$8:$D$32,$S16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="n"/>
+      <c r="B17" s="23" t="n"/>
+      <c r="C17" s="40" t="n"/>
+      <c r="D17" s="40" t="n"/>
+      <c r="E17" s="41" t="n"/>
+      <c r="F17" s="25">
+        <f>IFERROR($E17/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+      <c r="S17" t="n">
+        <v>720</v>
+      </c>
+      <c r="T17">
+        <f>SUMIFS($E$8:$E$32,$D$8:$D$32,$S17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="n"/>
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="40" t="n"/>
+      <c r="D18" s="40" t="n"/>
+      <c r="E18" s="41" t="n"/>
+      <c r="F18" s="25">
+        <f>IFERROR($E18/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+      <c r="S18" t="n">
+        <v>1800</v>
+      </c>
+      <c r="T18">
+        <f>SUMIFS($E$8:$E$32,$D$8:$D$32,$S18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="n"/>
+      <c r="B19" s="23" t="n"/>
+      <c r="C19" s="40" t="n"/>
+      <c r="D19" s="40" t="n"/>
+      <c r="E19" s="41" t="n"/>
+      <c r="F19" s="25">
+        <f>IFERROR($E19/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="n"/>
+      <c r="B20" s="23" t="n"/>
+      <c r="C20" s="40" t="n"/>
+      <c r="D20" s="40" t="n"/>
+      <c r="E20" s="41" t="n"/>
+      <c r="F20" s="25">
+        <f>IFERROR($E20/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="n"/>
+      <c r="B21" s="23" t="n"/>
+      <c r="C21" s="40" t="n"/>
+      <c r="D21" s="40" t="n"/>
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="25">
+        <f>IFERROR($E21/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="23" t="n"/>
+      <c r="C22" s="40" t="n"/>
+      <c r="D22" s="40" t="n"/>
+      <c r="E22" s="41" t="n"/>
+      <c r="F22" s="25">
+        <f>IFERROR($E22/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="n"/>
+      <c r="B23" s="23" t="n"/>
+      <c r="C23" s="40" t="n"/>
+      <c r="D23" s="40" t="n"/>
+      <c r="E23" s="41" t="n"/>
+      <c r="F23" s="25">
+        <f>IFERROR($E23/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="n"/>
+      <c r="B24" s="23" t="n"/>
+      <c r="C24" s="40" t="n"/>
+      <c r="D24" s="40" t="n"/>
+      <c r="E24" s="41" t="n"/>
+      <c r="F24" s="25">
+        <f>IFERROR($E24/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="n"/>
+      <c r="B25" s="23" t="n"/>
+      <c r="C25" s="40" t="n"/>
+      <c r="D25" s="40" t="n"/>
+      <c r="E25" s="41" t="n"/>
+      <c r="F25" s="25">
+        <f>IFERROR($E25/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="n"/>
+      <c r="B26" s="23" t="n"/>
+      <c r="C26" s="40" t="n"/>
+      <c r="D26" s="40" t="n"/>
+      <c r="E26" s="41" t="n"/>
+      <c r="F26" s="25">
+        <f>IFERROR($E26/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="n"/>
+      <c r="B27" s="23" t="n"/>
+      <c r="C27" s="40" t="n"/>
+      <c r="D27" s="40" t="n"/>
+      <c r="E27" s="41" t="n"/>
+      <c r="F27" s="25">
+        <f>IFERROR($E27/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="23" t="n"/>
+      <c r="C28" s="40" t="n"/>
+      <c r="D28" s="40" t="n"/>
+      <c r="E28" s="41" t="n"/>
+      <c r="F28" s="25">
+        <f>IFERROR($E28/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="n"/>
+      <c r="B29" s="23" t="n"/>
+      <c r="C29" s="40" t="n"/>
+      <c r="D29" s="40" t="n"/>
+      <c r="E29" s="41" t="n"/>
+      <c r="F29" s="25">
+        <f>IFERROR($E29/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="23" t="n"/>
+      <c r="B30" s="23" t="n"/>
+      <c r="C30" s="40" t="n"/>
+      <c r="D30" s="40" t="n"/>
+      <c r="E30" s="41" t="n"/>
+      <c r="F30" s="25">
+        <f>IFERROR($E30/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="n"/>
+      <c r="B31" s="23" t="n"/>
+      <c r="C31" s="40" t="n"/>
+      <c r="D31" s="40" t="n"/>
+      <c r="E31" s="41" t="n"/>
+      <c r="F31" s="25">
+        <f>IFERROR($E31/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="23" t="n"/>
+      <c r="B32" s="23" t="n"/>
+      <c r="C32" s="40" t="n"/>
+      <c r="D32" s="40" t="n"/>
+      <c r="E32" s="41" t="n"/>
+      <c r="F32" s="25">
+        <f>IFERROR($E32/SUM($E$8:$E$32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="28" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B33" s="29" t="n"/>
+      <c r="C33" s="29" t="n"/>
+      <c r="D33" s="29" t="n"/>
+      <c r="E33" s="42">
+        <f>SUM(E8:E32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="43">
+        <f>SUM(F8:F32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>OTIMIZAÇÕES REALIZADAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="44" t="n"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="44" t="n"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="44" t="n"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="44" t="n"/>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="44" t="n"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>RACIONAL POR MOVIMENTAÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Racional (objetivo e justificativa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="45" t="n"/>
+      <c r="B46" s="44" t="n"/>
+    </row>
+    <row r="47" ht="32" customHeight="1">
+      <c r="A47" s="45" t="n"/>
+      <c r="B47" s="44" t="n"/>
+    </row>
+    <row r="48" ht="32" customHeight="1">
+      <c r="A48" s="45" t="n"/>
+      <c r="B48" s="44" t="n"/>
+    </row>
+    <row r="49" ht="32" customHeight="1">
+      <c r="A49" s="45" t="n"/>
+      <c r="B49" s="44" t="n"/>
+    </row>
+    <row r="50" ht="32" customHeight="1">
+      <c r="A50" s="45" t="n"/>
+      <c r="B50" s="44" t="n"/>
+    </row>
+    <row r="51" ht="32" customHeight="1">
+      <c r="A51" s="45" t="n"/>
+      <c r="B51" s="44" t="n"/>
+    </row>
+    <row r="52" ht="32" customHeight="1">
+      <c r="A52" s="45" t="n"/>
+      <c r="B52" s="44" t="n"/>
+    </row>
+    <row r="53" ht="32" customHeight="1">
+      <c r="A53" s="45" t="n"/>
+      <c r="B53" s="44" t="n"/>
+    </row>
+    <row r="54" ht="32" customHeight="1">
+      <c r="A54" s="45" t="n"/>
+      <c r="B54" s="44" t="n"/>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="45" t="n"/>
+      <c r="B55" s="44" t="n"/>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
+        <is>
+          <t>COMPARATIVO: ATUAL x SUGERIDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>% Atual</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Classe</t>
+          <t>% Sugerido</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Investimento sugerido</t>
+          <t>Saldo Atual (R$)</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Valor (R$)</t>
+          <t>Valor Sugerido (R$)</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6">
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Diferença (R$)</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Ação</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6">
         <f>'Carteira do Cliente'!A11</f>
         <v/>
       </c>
-      <c r="B8" s="24">
+      <c r="B59" s="25">
+        <f>'Carteira do Cliente'!D11</f>
+        <v/>
+      </c>
+      <c r="C59" s="25">
+        <f>IFERROR($E59/SUM($E$8:$E$32),0)</f>
+        <v/>
+      </c>
+      <c r="D59" s="24">
         <f>'Carteira do Cliente'!C11</f>
         <v/>
       </c>
-      <c r="C8" s="25">
-        <f>'Carteira do Cliente'!D11</f>
-        <v/>
-      </c>
-      <c r="E8" s="23" t="n"/>
-      <c r="F8" s="23" t="n"/>
-      <c r="G8" s="38" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4">
+      <c r="E59" s="24">
+        <f>SUMIFS($E$8:$E$32,$A$8:$A$32,$A59)</f>
+        <v/>
+      </c>
+      <c r="F59" s="24">
+        <f>$E59-$D59</f>
+        <v/>
+      </c>
+      <c r="G59" s="6">
+        <f>IF(AND($D59=0,$E59=0),"",IF(ROUND($F59,2)&gt;0,"Aumentar",IF(ROUND($F59,2)&lt;0,"Reduzir","Manter")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4">
         <f>'Carteira do Cliente'!A12</f>
         <v/>
       </c>
-      <c r="B9" s="26">
+      <c r="B60" s="27">
+        <f>'Carteira do Cliente'!D12</f>
+        <v/>
+      </c>
+      <c r="C60" s="27">
+        <f>IFERROR($E60/SUM($E$8:$E$32),0)</f>
+        <v/>
+      </c>
+      <c r="D60" s="26">
         <f>'Carteira do Cliente'!C12</f>
         <v/>
       </c>
-      <c r="C9" s="27">
-        <f>'Carteira do Cliente'!D12</f>
-        <v/>
-      </c>
-      <c r="E9" s="23" t="n"/>
-      <c r="F9" s="23" t="n"/>
-      <c r="G9" s="38" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6">
+      <c r="E60" s="26">
+        <f>SUMIFS($E$8:$E$32,$A$8:$A$32,$A60)</f>
+        <v/>
+      </c>
+      <c r="F60" s="26">
+        <f>$E60-$D60</f>
+        <v/>
+      </c>
+      <c r="G60" s="4">
+        <f>IF(AND($D60=0,$E60=0),"",IF(ROUND($F60,2)&gt;0,"Aumentar",IF(ROUND($F60,2)&lt;0,"Reduzir","Manter")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6">
         <f>'Carteira do Cliente'!A13</f>
         <v/>
       </c>
-      <c r="B10" s="24">
+      <c r="B61" s="25">
+        <f>'Carteira do Cliente'!D13</f>
+        <v/>
+      </c>
+      <c r="C61" s="25">
+        <f>IFERROR($E61/SUM($E$8:$E$32),0)</f>
+        <v/>
+      </c>
+      <c r="D61" s="24">
         <f>'Carteira do Cliente'!C13</f>
         <v/>
       </c>
-      <c r="C10" s="25">
-        <f>'Carteira do Cliente'!D13</f>
-        <v/>
-      </c>
-      <c r="E10" s="23" t="n"/>
-      <c r="F10" s="23" t="n"/>
-      <c r="G10" s="38" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4">
+      <c r="E61" s="24">
+        <f>SUMIFS($E$8:$E$32,$A$8:$A$32,$A61)</f>
+        <v/>
+      </c>
+      <c r="F61" s="24">
+        <f>$E61-$D61</f>
+        <v/>
+      </c>
+      <c r="G61" s="6">
+        <f>IF(AND($D61=0,$E61=0),"",IF(ROUND($F61,2)&gt;0,"Aumentar",IF(ROUND($F61,2)&lt;0,"Reduzir","Manter")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4">
         <f>'Carteira do Cliente'!A14</f>
         <v/>
       </c>
-      <c r="B11" s="26">
+      <c r="B62" s="27">
+        <f>'Carteira do Cliente'!D14</f>
+        <v/>
+      </c>
+      <c r="C62" s="27">
+        <f>IFERROR($E62/SUM($E$8:$E$32),0)</f>
+        <v/>
+      </c>
+      <c r="D62" s="26">
         <f>'Carteira do Cliente'!C14</f>
         <v/>
       </c>
-      <c r="C11" s="27">
-        <f>'Carteira do Cliente'!D14</f>
-        <v/>
-      </c>
-      <c r="E11" s="23" t="n"/>
-      <c r="F11" s="23" t="n"/>
-      <c r="G11" s="38" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6">
+      <c r="E62" s="26">
+        <f>SUMIFS($E$8:$E$32,$A$8:$A$32,$A62)</f>
+        <v/>
+      </c>
+      <c r="F62" s="26">
+        <f>$E62-$D62</f>
+        <v/>
+      </c>
+      <c r="G62" s="4">
+        <f>IF(AND($D62=0,$E62=0),"",IF(ROUND($F62,2)&gt;0,"Aumentar",IF(ROUND($F62,2)&lt;0,"Reduzir","Manter")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6">
         <f>'Carteira do Cliente'!A15</f>
         <v/>
       </c>
-      <c r="B12" s="24">
+      <c r="B63" s="25">
+        <f>'Carteira do Cliente'!D15</f>
+        <v/>
+      </c>
+      <c r="C63" s="25">
+        <f>IFERROR($E63/SUM($E$8:$E$32),0)</f>
+        <v/>
+      </c>
+      <c r="D63" s="24">
         <f>'Carteira do Cliente'!C15</f>
         <v/>
       </c>
-      <c r="C12" s="25">
-        <f>'Carteira do Cliente'!D15</f>
-        <v/>
-      </c>
-      <c r="E12" s="23" t="n"/>
-      <c r="F12" s="23" t="n"/>
-      <c r="G12" s="38" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4">
+      <c r="E63" s="24">
+        <f>SUMIFS($E$8:$E$32,$A$8:$A$32,$A63)</f>
+        <v/>
+      </c>
+      <c r="F63" s="24">
+        <f>$E63-$D63</f>
+        <v/>
+      </c>
+      <c r="G63" s="6">
+        <f>IF(AND($D63=0,$E63=0),"",IF(ROUND($F63,2)&gt;0,"Aumentar",IF(ROUND($F63,2)&lt;0,"Reduzir","Manter")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4">
         <f>'Carteira do Cliente'!A16</f>
         <v/>
       </c>
-      <c r="B13" s="26">
+      <c r="B64" s="27">
+        <f>'Carteira do Cliente'!D16</f>
+        <v/>
+      </c>
+      <c r="C64" s="27">
+        <f>IFERROR($E64/SUM($E$8:$E$32),0)</f>
+        <v/>
+      </c>
+      <c r="D64" s="26">
         <f>'Carteira do Cliente'!C16</f>
         <v/>
       </c>
-      <c r="C13" s="27">
-        <f>'Carteira do Cliente'!D16</f>
-        <v/>
-      </c>
-      <c r="E13" s="23" t="n"/>
-      <c r="F13" s="23" t="n"/>
-      <c r="G13" s="38" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6">
+      <c r="E64" s="26">
+        <f>SUMIFS($E$8:$E$32,$A$8:$A$32,$A64)</f>
+        <v/>
+      </c>
+      <c r="F64" s="26">
+        <f>$E64-$D64</f>
+        <v/>
+      </c>
+      <c r="G64" s="4">
+        <f>IF(AND($D64=0,$E64=0),"",IF(ROUND($F64,2)&gt;0,"Aumentar",IF(ROUND($F64,2)&lt;0,"Reduzir","Manter")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6">
         <f>'Carteira do Cliente'!A17</f>
         <v/>
       </c>
-      <c r="B14" s="24">
+      <c r="B65" s="25">
+        <f>'Carteira do Cliente'!D17</f>
+        <v/>
+      </c>
+      <c r="C65" s="25">
+        <f>IFERROR($E65/SUM($E$8:$E$32),0)</f>
+        <v/>
+      </c>
+      <c r="D65" s="24">
         <f>'Carteira do Cliente'!C17</f>
         <v/>
       </c>
-      <c r="C14" s="25">
-        <f>'Carteira do Cliente'!D17</f>
-        <v/>
-      </c>
-      <c r="E14" s="23" t="n"/>
-      <c r="F14" s="23" t="n"/>
-      <c r="G14" s="38" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4">
+      <c r="E65" s="24">
+        <f>SUMIFS($E$8:$E$32,$A$8:$A$32,$A65)</f>
+        <v/>
+      </c>
+      <c r="F65" s="24">
+        <f>$E65-$D65</f>
+        <v/>
+      </c>
+      <c r="G65" s="6">
+        <f>IF(AND($D65=0,$E65=0),"",IF(ROUND($F65,2)&gt;0,"Aumentar",IF(ROUND($F65,2)&lt;0,"Reduzir","Manter")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4">
         <f>'Carteira do Cliente'!A18</f>
         <v/>
       </c>
-      <c r="B15" s="26">
+      <c r="B66" s="27">
+        <f>'Carteira do Cliente'!D18</f>
+        <v/>
+      </c>
+      <c r="C66" s="27">
+        <f>IFERROR($E66/SUM($E$8:$E$32),0)</f>
+        <v/>
+      </c>
+      <c r="D66" s="26">
         <f>'Carteira do Cliente'!C18</f>
         <v/>
       </c>
-      <c r="C15" s="27">
-        <f>'Carteira do Cliente'!D18</f>
-        <v/>
-      </c>
-      <c r="E15" s="23" t="n"/>
-      <c r="F15" s="23" t="n"/>
-      <c r="G15" s="38" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="E66" s="26">
+        <f>SUMIFS($E$8:$E$32,$A$8:$A$32,$A66)</f>
+        <v/>
+      </c>
+      <c r="F66" s="26">
+        <f>$E66-$D66</f>
+        <v/>
+      </c>
+      <c r="G66" s="4">
+        <f>IF(AND($D66=0,$E66=0),"",IF(ROUND($F66,2)&gt;0,"Aumentar",IF(ROUND($F66,2)&lt;0,"Reduzir","Manter")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="28" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B16" s="39">
-        <f>SUM(B8:B15)</f>
-        <v/>
-      </c>
-      <c r="C16" s="40">
-        <f>SUM(C8:C15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="23" t="n"/>
-      <c r="F16" s="23" t="n"/>
-      <c r="G16" s="38" t="n"/>
-    </row>
-    <row r="17">
-      <c r="E17" s="23" t="n"/>
-      <c r="F17" s="23" t="n"/>
-      <c r="G17" s="38" t="n"/>
-    </row>
-    <row r="18">
-      <c r="E18" s="23" t="n"/>
-      <c r="F18" s="23" t="n"/>
-      <c r="G18" s="38" t="n"/>
-    </row>
-    <row r="19">
-      <c r="E19" s="23" t="n"/>
-      <c r="F19" s="23" t="n"/>
-      <c r="G19" s="38" t="n"/>
-    </row>
-    <row r="20">
-      <c r="E20" s="23" t="n"/>
-      <c r="F20" s="23" t="n"/>
-      <c r="G20" s="38" t="n"/>
-    </row>
-    <row r="21">
-      <c r="E21" s="23" t="n"/>
-      <c r="F21" s="23" t="n"/>
-      <c r="G21" s="38" t="n"/>
-    </row>
-    <row r="22">
-      <c r="E22" s="23" t="n"/>
-      <c r="F22" s="23" t="n"/>
-      <c r="G22" s="38" t="n"/>
-    </row>
-    <row r="23">
-      <c r="E23" s="23" t="n"/>
-      <c r="F23" s="23" t="n"/>
-      <c r="G23" s="38" t="n"/>
-    </row>
-    <row r="24">
-      <c r="E24" s="23" t="n"/>
-      <c r="F24" s="23" t="n"/>
-      <c r="G24" s="38" t="n"/>
-    </row>
-    <row r="25">
-      <c r="E25" s="23" t="n"/>
-      <c r="F25" s="23" t="n"/>
-      <c r="G25" s="38" t="n"/>
-    </row>
-    <row r="26">
-      <c r="E26" s="23" t="n"/>
-      <c r="F26" s="23" t="n"/>
-      <c r="G26" s="38" t="n"/>
-    </row>
-    <row r="27">
-      <c r="E27" s="23" t="n"/>
-      <c r="F27" s="23" t="n"/>
-      <c r="G27" s="38" t="n"/>
-    </row>
-    <row r="28">
-      <c r="E28" s="23" t="n"/>
-      <c r="F28" s="23" t="n"/>
-      <c r="G28" s="38" t="n"/>
-    </row>
-    <row r="29">
-      <c r="E29" s="23" t="n"/>
-      <c r="F29" s="23" t="n"/>
-      <c r="G29" s="38" t="n"/>
-    </row>
-    <row r="30">
-      <c r="E30" s="23" t="n"/>
-      <c r="F30" s="23" t="n"/>
-      <c r="G30" s="38" t="n"/>
-    </row>
-    <row r="31">
-      <c r="E31" s="23" t="n"/>
-      <c r="F31" s="23" t="n"/>
-      <c r="G31" s="38" t="n"/>
-    </row>
-    <row r="32">
-      <c r="E32" s="23" t="n"/>
-      <c r="F32" s="23" t="n"/>
-      <c r="G32" s="38" t="n"/>
-    </row>
-    <row r="33">
-      <c r="F33" s="41" t="inlineStr">
-        <is>
-          <t>TOTAL SUGERIDO</t>
-        </is>
-      </c>
-      <c r="G33" s="30">
-        <f>SUM(G8:G32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="22" t="inlineStr">
-        <is>
-          <t>COMPARATIVO: ATUAL x SUGERIDA</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Classe</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>% Atual</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>% Sugerido</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Saldo Atual (R$)</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Valor Sugerido (R$)</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Diferença (R$)</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>Ação</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="6">
-        <f>'Carteira do Cliente'!A11</f>
-        <v/>
-      </c>
-      <c r="B38" s="25">
-        <f>'Carteira do Cliente'!D11</f>
-        <v/>
-      </c>
-      <c r="C38" s="25">
-        <f>IFERROR($E38/$G$33,0)</f>
-        <v/>
-      </c>
-      <c r="D38" s="24">
-        <f>'Carteira do Cliente'!C11</f>
-        <v/>
-      </c>
-      <c r="E38" s="24">
-        <f>SUMIFS($G$8:$G$32,$E$8:$E$32,$A38)</f>
-        <v/>
-      </c>
-      <c r="F38" s="24">
-        <f>$E38-$D38</f>
-        <v/>
-      </c>
-      <c r="G38" s="6">
-        <f>IF(AND($D38=0,$E38=0),"",IF(ROUND($F38,2)&gt;0,"Aumentar",IF(ROUND($F38,2)&lt;0,"Reduzir","Manter")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4">
-        <f>'Carteira do Cliente'!A12</f>
-        <v/>
-      </c>
-      <c r="B39" s="27">
-        <f>'Carteira do Cliente'!D12</f>
-        <v/>
-      </c>
-      <c r="C39" s="27">
-        <f>IFERROR($E39/$G$33,0)</f>
-        <v/>
-      </c>
-      <c r="D39" s="26">
-        <f>'Carteira do Cliente'!C12</f>
-        <v/>
-      </c>
-      <c r="E39" s="26">
-        <f>SUMIFS($G$8:$G$32,$E$8:$E$32,$A39)</f>
-        <v/>
-      </c>
-      <c r="F39" s="26">
-        <f>$E39-$D39</f>
-        <v/>
-      </c>
-      <c r="G39" s="4">
-        <f>IF(AND($D39=0,$E39=0),"",IF(ROUND($F39,2)&gt;0,"Aumentar",IF(ROUND($F39,2)&lt;0,"Reduzir","Manter")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6">
-        <f>'Carteira do Cliente'!A13</f>
-        <v/>
-      </c>
-      <c r="B40" s="25">
-        <f>'Carteira do Cliente'!D13</f>
-        <v/>
-      </c>
-      <c r="C40" s="25">
-        <f>IFERROR($E40/$G$33,0)</f>
-        <v/>
-      </c>
-      <c r="D40" s="24">
-        <f>'Carteira do Cliente'!C13</f>
-        <v/>
-      </c>
-      <c r="E40" s="24">
-        <f>SUMIFS($G$8:$G$32,$E$8:$E$32,$A40)</f>
-        <v/>
-      </c>
-      <c r="F40" s="24">
-        <f>$E40-$D40</f>
-        <v/>
-      </c>
-      <c r="G40" s="6">
-        <f>IF(AND($D40=0,$E40=0),"",IF(ROUND($F40,2)&gt;0,"Aumentar",IF(ROUND($F40,2)&lt;0,"Reduzir","Manter")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4">
-        <f>'Carteira do Cliente'!A14</f>
-        <v/>
-      </c>
-      <c r="B41" s="27">
-        <f>'Carteira do Cliente'!D14</f>
-        <v/>
-      </c>
-      <c r="C41" s="27">
-        <f>IFERROR($E41/$G$33,0)</f>
-        <v/>
-      </c>
-      <c r="D41" s="26">
-        <f>'Carteira do Cliente'!C14</f>
-        <v/>
-      </c>
-      <c r="E41" s="26">
-        <f>SUMIFS($G$8:$G$32,$E$8:$E$32,$A41)</f>
-        <v/>
-      </c>
-      <c r="F41" s="26">
-        <f>$E41-$D41</f>
-        <v/>
-      </c>
-      <c r="G41" s="4">
-        <f>IF(AND($D41=0,$E41=0),"",IF(ROUND($F41,2)&gt;0,"Aumentar",IF(ROUND($F41,2)&lt;0,"Reduzir","Manter")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6">
-        <f>'Carteira do Cliente'!A15</f>
-        <v/>
-      </c>
-      <c r="B42" s="25">
-        <f>'Carteira do Cliente'!D15</f>
-        <v/>
-      </c>
-      <c r="C42" s="25">
-        <f>IFERROR($E42/$G$33,0)</f>
-        <v/>
-      </c>
-      <c r="D42" s="24">
-        <f>'Carteira do Cliente'!C15</f>
-        <v/>
-      </c>
-      <c r="E42" s="24">
-        <f>SUMIFS($G$8:$G$32,$E$8:$E$32,$A42)</f>
-        <v/>
-      </c>
-      <c r="F42" s="24">
-        <f>$E42-$D42</f>
-        <v/>
-      </c>
-      <c r="G42" s="6">
-        <f>IF(AND($D42=0,$E42=0),"",IF(ROUND($F42,2)&gt;0,"Aumentar",IF(ROUND($F42,2)&lt;0,"Reduzir","Manter")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4">
-        <f>'Carteira do Cliente'!A16</f>
-        <v/>
-      </c>
-      <c r="B43" s="27">
-        <f>'Carteira do Cliente'!D16</f>
-        <v/>
-      </c>
-      <c r="C43" s="27">
-        <f>IFERROR($E43/$G$33,0)</f>
-        <v/>
-      </c>
-      <c r="D43" s="26">
-        <f>'Carteira do Cliente'!C16</f>
-        <v/>
-      </c>
-      <c r="E43" s="26">
-        <f>SUMIFS($G$8:$G$32,$E$8:$E$32,$A43)</f>
-        <v/>
-      </c>
-      <c r="F43" s="26">
-        <f>$E43-$D43</f>
-        <v/>
-      </c>
-      <c r="G43" s="4">
-        <f>IF(AND($D43=0,$E43=0),"",IF(ROUND($F43,2)&gt;0,"Aumentar",IF(ROUND($F43,2)&lt;0,"Reduzir","Manter")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="6">
-        <f>'Carteira do Cliente'!A17</f>
-        <v/>
-      </c>
-      <c r="B44" s="25">
-        <f>'Carteira do Cliente'!D17</f>
-        <v/>
-      </c>
-      <c r="C44" s="25">
-        <f>IFERROR($E44/$G$33,0)</f>
-        <v/>
-      </c>
-      <c r="D44" s="24">
-        <f>'Carteira do Cliente'!C17</f>
-        <v/>
-      </c>
-      <c r="E44" s="24">
-        <f>SUMIFS($G$8:$G$32,$E$8:$E$32,$A44)</f>
-        <v/>
-      </c>
-      <c r="F44" s="24">
-        <f>$E44-$D44</f>
-        <v/>
-      </c>
-      <c r="G44" s="6">
-        <f>IF(AND($D44=0,$E44=0),"",IF(ROUND($F44,2)&gt;0,"Aumentar",IF(ROUND($F44,2)&lt;0,"Reduzir","Manter")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4">
-        <f>'Carteira do Cliente'!A18</f>
-        <v/>
-      </c>
-      <c r="B45" s="27">
-        <f>'Carteira do Cliente'!D18</f>
-        <v/>
-      </c>
-      <c r="C45" s="27">
-        <f>IFERROR($E45/$G$33,0)</f>
-        <v/>
-      </c>
-      <c r="D45" s="26">
-        <f>'Carteira do Cliente'!C18</f>
-        <v/>
-      </c>
-      <c r="E45" s="26">
-        <f>SUMIFS($G$8:$G$32,$E$8:$E$32,$A45)</f>
-        <v/>
-      </c>
-      <c r="F45" s="26">
-        <f>$E45-$D45</f>
-        <v/>
-      </c>
-      <c r="G45" s="4">
-        <f>IF(AND($D45=0,$E45=0),"",IF(ROUND($F45,2)&gt;0,"Aumentar",IF(ROUND($F45,2)&lt;0,"Reduzir","Manter")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="28" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D46" s="39">
-        <f>SUM(D38:D45)</f>
-        <v/>
-      </c>
-      <c r="E46" s="39">
-        <f>SUM(E38:E45)</f>
-        <v/>
-      </c>
-      <c r="F46" s="39">
-        <f>SUM(F38:F45)</f>
+      <c r="D67" s="42">
+        <f>SUM(D59:D66)</f>
+        <v/>
+      </c>
+      <c r="E67" s="42">
+        <f>SUM(E59:E66)</f>
+        <v/>
+      </c>
+      <c r="F67" s="42">
+        <f>SUM(F59:F66)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="E6:G6"/>
+  <mergeCells count="25">
+    <mergeCell ref="A40:N40"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="B49:N49"/>
+    <mergeCell ref="H3:N3"/>
+    <mergeCell ref="B55:N55"/>
+    <mergeCell ref="B51:N51"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="B45:N45"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B50:N50"/>
+    <mergeCell ref="A41:N41"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="A37:N37"/>
+    <mergeCell ref="B47:N47"/>
+    <mergeCell ref="B54:N54"/>
+    <mergeCell ref="B46:N46"/>
+    <mergeCell ref="H4:N4"/>
+    <mergeCell ref="B52:N52"/>
+    <mergeCell ref="B48:N48"/>
+    <mergeCell ref="A42:N42"/>
+    <mergeCell ref="A38:N38"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="B53:N53"/>
+    <mergeCell ref="A57:G57"/>
+    <mergeCell ref="A44:N44"/>
   </mergeCells>
-  <conditionalFormatting sqref="G38:G45">
+  <conditionalFormatting sqref="G59:G66">
     <cfRule type="expression" priority="1" dxfId="1">
-      <formula>$G38="Aumentar"</formula>
+      <formula>$G59="Aumentar"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>$G38="Reduzir"</formula>
+      <formula>$G59="Reduzir"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E8:E32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A8:A32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='Carteira do Cliente'!$A$11:$A$18</formula1>
     </dataValidation>
   </dataValidations>
@@ -29644,109 +30290,1663 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:J74"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PLANEJAMENTO FINANCEIRO &amp; APOSENTADORIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Cliente:</t>
+        </is>
+      </c>
+      <c r="B3" s="36">
+        <f>'Carteira do Cliente'!B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>INFORMAÇÕES GERAIS E PATRIMÔNIO ATUAL</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>INFLAÇÃO, CDI, ALÍQUOTA IR E TAXA NOMINAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Idade atual (anos)</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="n">
+        <v>51</v>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>Inflação anual projetada</t>
+        </is>
+      </c>
+      <c r="E6" s="47" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Idade de aposentadoria (anos)</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="n">
+        <v>64</v>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>Alíquota de IR (sobre rendimentos)</t>
+        </is>
+      </c>
+      <c r="E7" s="47" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Expectativa de vida (anos)</t>
+        </is>
+      </c>
+      <c r="B8" s="46" t="n">
+        <v>90</v>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>Taxa CDI anual</t>
+        </is>
+      </c>
+      <c r="E8" s="47" t="n">
+        <v>0.1065</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Horizonte de produção/acumulação (anos)</t>
+        </is>
+      </c>
+      <c r="B9" s="12">
+        <f>B7-B6</f>
+        <v/>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>% do CDI esperado (rentabilidade)</t>
+        </is>
+      </c>
+      <c r="E9" s="47" t="n">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Patrimônio líquido disponível (R$)</t>
+        </is>
+      </c>
+      <c r="B10" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>Taxa nominal anual bruta (calc)</t>
+        </is>
+      </c>
+      <c r="E10" s="49">
+        <f>E8*E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Aplicação mensal (Prev + Meta) (R$)</t>
+        </is>
+      </c>
+      <c r="B11" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>Taxa nominal anual líquida (calc)</t>
+        </is>
+      </c>
+      <c r="E11" s="49">
+        <f>E10*(1-E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>PREMISSAS DE APOSENTADORIA</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>TAXA DE JUROS REAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Renda desejada na aposentadoria (R$ / mês)</t>
+        </is>
+      </c>
+      <c r="B14" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>Taxa real anual bruta</t>
+        </is>
+      </c>
+      <c r="E14" s="49">
+        <f>(1+E10)/(1+E6)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Renda projetada do INSS (R$ / mês)</t>
+        </is>
+      </c>
+      <c r="B15" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Taxa real anual líquida</t>
+        </is>
+      </c>
+      <c r="E15" s="49">
+        <f>(1+E11)/(1+E6)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Outras fontes de renda (R$ / mês)</t>
+        </is>
+      </c>
+      <c r="B16" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Taxa real anual líquida pós-aposentadoria</t>
+        </is>
+      </c>
+      <c r="E16" s="47" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Renda a sustentar pelo patrimônio (R$ / mês)</t>
+        </is>
+      </c>
+      <c r="B17" s="14">
+        <f>MAX(0,B14-B15-B16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Taxa real mensal líquida pós-aposentadoria</t>
+        </is>
+      </c>
+      <c r="E17" s="50">
+        <f>(1+E16)^(1/12)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Renda a sustentar pelo patrimônio (R$ / ano)</t>
+        </is>
+      </c>
+      <c r="B18" s="14">
+        <f>B17*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>APOSENTADORIA — VIVER DE RENDA (preservando)</t>
+        </is>
+      </c>
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>APOSENTADORIA — CONSUMO COM SUCESSÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Patrimônio necessário na aposentadoria</t>
+        </is>
+      </c>
+      <c r="B21" s="20">
+        <f>IFERROR(B18/E16,0)</f>
+        <v/>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>Patrimônio de sucessão desejado (R$)</t>
+        </is>
+      </c>
+      <c r="E21" s="48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Parcela mensal necessária a aplicar</t>
+        </is>
+      </c>
+      <c r="B22" s="20">
+        <f>IFERROR(-PMT(E17,B9*12,-B10,B21),0)</f>
+        <v/>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>Patrimônio necessário na aposentadoria</t>
+        </is>
+      </c>
+      <c r="E22" s="20">
+        <f>IFERROR(PV(E16,B8-B7,-B18,-E21),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>Parcela mensal necessária a aplicar</t>
+        </is>
+      </c>
+      <c r="E23" s="20">
+        <f>IFERROR(-PMT(E17,B9*12,-B10,E22),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>OBJETIVOS DE VIDA (1-6 anos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Projeto</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Valor hoje (R$)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Acumulação projetada (R$)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Anos</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Projetos 1-2 anos</t>
+        </is>
+      </c>
+      <c r="B27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="20">
+        <f>B27*(1+E10)^E27</f>
+        <v/>
+      </c>
+      <c r="E27" s="51" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>Projetos 3-4 anos</t>
+        </is>
+      </c>
+      <c r="B28" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="20">
+        <f>B28*(1+E10)^E28</f>
+        <v/>
+      </c>
+      <c r="E28" s="51" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Projetos 5-6 anos</t>
+        </is>
+      </c>
+      <c r="B29" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="20">
+        <f>B29*(1+E10)^E29</f>
+        <v/>
+      </c>
+      <c r="E29" s="51" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Total de Projetos e Acumulação</t>
+        </is>
+      </c>
+      <c r="B30" s="20">
+        <f>SUM(B27:B29)</f>
+        <v/>
+      </c>
+      <c r="D30" s="20">
+        <f>SUM(D27:D29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="G33" s="22" t="inlineStr">
+        <is>
+          <t>PROJEÇÃO PATRIMONIAL (em R$ reais de hoje)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Idade</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Saldo Real</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Viver de Renda</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="G35" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="52">
+        <f>B6+G35</f>
+        <v/>
+      </c>
+      <c r="I35" s="53">
+        <f>B10</f>
+        <v/>
+      </c>
+      <c r="J35" s="53">
+        <f>IF(H35&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="G36" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="54">
+        <f>B6+G36</f>
+        <v/>
+      </c>
+      <c r="I36" s="55">
+        <f>IF(H36&lt;=B7,I35*(1+E15)+B11*12,MAX(0,I35*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J36" s="55">
+        <f>IF(H36&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="G37" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" s="52">
+        <f>B6+G37</f>
+        <v/>
+      </c>
+      <c r="I37" s="53">
+        <f>IF(H37&lt;=B7,I36*(1+E15)+B11*12,MAX(0,I36*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J37" s="53">
+        <f>IF(H37&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="G38" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="H38" s="54">
+        <f>B6+G38</f>
+        <v/>
+      </c>
+      <c r="I38" s="55">
+        <f>IF(H38&lt;=B7,I37*(1+E15)+B11*12,MAX(0,I37*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J38" s="55">
+        <f>IF(H38&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="G39" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="H39" s="52">
+        <f>B6+G39</f>
+        <v/>
+      </c>
+      <c r="I39" s="53">
+        <f>IF(H39&lt;=B7,I38*(1+E15)+B11*12,MAX(0,I38*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J39" s="53">
+        <f>IF(H39&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="G40" s="54" t="n">
+        <v>5</v>
+      </c>
+      <c r="H40" s="54">
+        <f>B6+G40</f>
+        <v/>
+      </c>
+      <c r="I40" s="55">
+        <f>IF(H40&lt;=B7,I39*(1+E15)+B11*12,MAX(0,I39*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J40" s="55">
+        <f>IF(H40&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="G41" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="H41" s="52">
+        <f>B6+G41</f>
+        <v/>
+      </c>
+      <c r="I41" s="53">
+        <f>IF(H41&lt;=B7,I40*(1+E15)+B11*12,MAX(0,I40*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J41" s="53">
+        <f>IF(H41&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="G42" s="54" t="n">
+        <v>7</v>
+      </c>
+      <c r="H42" s="54">
+        <f>B6+G42</f>
+        <v/>
+      </c>
+      <c r="I42" s="55">
+        <f>IF(H42&lt;=B7,I41*(1+E15)+B11*12,MAX(0,I41*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J42" s="55">
+        <f>IF(H42&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="G43" s="52" t="n">
+        <v>8</v>
+      </c>
+      <c r="H43" s="52">
+        <f>B6+G43</f>
+        <v/>
+      </c>
+      <c r="I43" s="53">
+        <f>IF(H43&lt;=B7,I42*(1+E15)+B11*12,MAX(0,I42*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J43" s="53">
+        <f>IF(H43&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="G44" s="54" t="n">
+        <v>9</v>
+      </c>
+      <c r="H44" s="54">
+        <f>B6+G44</f>
+        <v/>
+      </c>
+      <c r="I44" s="55">
+        <f>IF(H44&lt;=B7,I43*(1+E15)+B11*12,MAX(0,I43*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J44" s="55">
+        <f>IF(H44&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="G45" s="52" t="n">
+        <v>10</v>
+      </c>
+      <c r="H45" s="52">
+        <f>B6+G45</f>
+        <v/>
+      </c>
+      <c r="I45" s="53">
+        <f>IF(H45&lt;=B7,I44*(1+E15)+B11*12,MAX(0,I44*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J45" s="53">
+        <f>IF(H45&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="G46" s="54" t="n">
+        <v>11</v>
+      </c>
+      <c r="H46" s="54">
+        <f>B6+G46</f>
+        <v/>
+      </c>
+      <c r="I46" s="55">
+        <f>IF(H46&lt;=B7,I45*(1+E15)+B11*12,MAX(0,I45*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J46" s="55">
+        <f>IF(H46&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="G47" s="52" t="n">
+        <v>12</v>
+      </c>
+      <c r="H47" s="52">
+        <f>B6+G47</f>
+        <v/>
+      </c>
+      <c r="I47" s="53">
+        <f>IF(H47&lt;=B7,I46*(1+E15)+B11*12,MAX(0,I46*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J47" s="53">
+        <f>IF(H47&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="G48" s="54" t="n">
+        <v>13</v>
+      </c>
+      <c r="H48" s="54">
+        <f>B6+G48</f>
+        <v/>
+      </c>
+      <c r="I48" s="55">
+        <f>IF(H48&lt;=B7,I47*(1+E15)+B11*12,MAX(0,I47*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J48" s="55">
+        <f>IF(H48&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="G49" s="52" t="n">
+        <v>14</v>
+      </c>
+      <c r="H49" s="52">
+        <f>B6+G49</f>
+        <v/>
+      </c>
+      <c r="I49" s="53">
+        <f>IF(H49&lt;=B7,I48*(1+E15)+B11*12,MAX(0,I48*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J49" s="53">
+        <f>IF(H49&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="G50" s="54" t="n">
+        <v>15</v>
+      </c>
+      <c r="H50" s="54">
+        <f>B6+G50</f>
+        <v/>
+      </c>
+      <c r="I50" s="55">
+        <f>IF(H50&lt;=B7,I49*(1+E15)+B11*12,MAX(0,I49*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J50" s="55">
+        <f>IF(H50&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="G51" s="52" t="n">
+        <v>16</v>
+      </c>
+      <c r="H51" s="52">
+        <f>B6+G51</f>
+        <v/>
+      </c>
+      <c r="I51" s="53">
+        <f>IF(H51&lt;=B7,I50*(1+E15)+B11*12,MAX(0,I50*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J51" s="53">
+        <f>IF(H51&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="G52" s="54" t="n">
+        <v>17</v>
+      </c>
+      <c r="H52" s="54">
+        <f>B6+G52</f>
+        <v/>
+      </c>
+      <c r="I52" s="55">
+        <f>IF(H52&lt;=B7,I51*(1+E15)+B11*12,MAX(0,I51*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J52" s="55">
+        <f>IF(H52&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="G53" s="52" t="n">
+        <v>18</v>
+      </c>
+      <c r="H53" s="52">
+        <f>B6+G53</f>
+        <v/>
+      </c>
+      <c r="I53" s="53">
+        <f>IF(H53&lt;=B7,I52*(1+E15)+B11*12,MAX(0,I52*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J53" s="53">
+        <f>IF(H53&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="G54" s="54" t="n">
+        <v>19</v>
+      </c>
+      <c r="H54" s="54">
+        <f>B6+G54</f>
+        <v/>
+      </c>
+      <c r="I54" s="55">
+        <f>IF(H54&lt;=B7,I53*(1+E15)+B11*12,MAX(0,I53*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J54" s="55">
+        <f>IF(H54&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="G55" s="52" t="n">
+        <v>20</v>
+      </c>
+      <c r="H55" s="52">
+        <f>B6+G55</f>
+        <v/>
+      </c>
+      <c r="I55" s="53">
+        <f>IF(H55&lt;=B7,I54*(1+E15)+B11*12,MAX(0,I54*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J55" s="53">
+        <f>IF(H55&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="G56" s="54" t="n">
+        <v>21</v>
+      </c>
+      <c r="H56" s="54">
+        <f>B6+G56</f>
+        <v/>
+      </c>
+      <c r="I56" s="55">
+        <f>IF(H56&lt;=B7,I55*(1+E15)+B11*12,MAX(0,I55*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J56" s="55">
+        <f>IF(H56&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="G57" s="52" t="n">
+        <v>22</v>
+      </c>
+      <c r="H57" s="52">
+        <f>B6+G57</f>
+        <v/>
+      </c>
+      <c r="I57" s="53">
+        <f>IF(H57&lt;=B7,I56*(1+E15)+B11*12,MAX(0,I56*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J57" s="53">
+        <f>IF(H57&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="G58" s="54" t="n">
+        <v>23</v>
+      </c>
+      <c r="H58" s="54">
+        <f>B6+G58</f>
+        <v/>
+      </c>
+      <c r="I58" s="55">
+        <f>IF(H58&lt;=B7,I57*(1+E15)+B11*12,MAX(0,I57*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J58" s="55">
+        <f>IF(H58&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="G59" s="52" t="n">
+        <v>24</v>
+      </c>
+      <c r="H59" s="52">
+        <f>B6+G59</f>
+        <v/>
+      </c>
+      <c r="I59" s="53">
+        <f>IF(H59&lt;=B7,I58*(1+E15)+B11*12,MAX(0,I58*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J59" s="53">
+        <f>IF(H59&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="G60" s="54" t="n">
+        <v>25</v>
+      </c>
+      <c r="H60" s="54">
+        <f>B6+G60</f>
+        <v/>
+      </c>
+      <c r="I60" s="55">
+        <f>IF(H60&lt;=B7,I59*(1+E15)+B11*12,MAX(0,I59*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J60" s="55">
+        <f>IF(H60&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="G61" s="52" t="n">
+        <v>26</v>
+      </c>
+      <c r="H61" s="52">
+        <f>B6+G61</f>
+        <v/>
+      </c>
+      <c r="I61" s="53">
+        <f>IF(H61&lt;=B7,I60*(1+E15)+B11*12,MAX(0,I60*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J61" s="53">
+        <f>IF(H61&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="G62" s="54" t="n">
+        <v>27</v>
+      </c>
+      <c r="H62" s="54">
+        <f>B6+G62</f>
+        <v/>
+      </c>
+      <c r="I62" s="55">
+        <f>IF(H62&lt;=B7,I61*(1+E15)+B11*12,MAX(0,I61*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J62" s="55">
+        <f>IF(H62&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="G63" s="52" t="n">
+        <v>28</v>
+      </c>
+      <c r="H63" s="52">
+        <f>B6+G63</f>
+        <v/>
+      </c>
+      <c r="I63" s="53">
+        <f>IF(H63&lt;=B7,I62*(1+E15)+B11*12,MAX(0,I62*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J63" s="53">
+        <f>IF(H63&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="G64" s="54" t="n">
+        <v>29</v>
+      </c>
+      <c r="H64" s="54">
+        <f>B6+G64</f>
+        <v/>
+      </c>
+      <c r="I64" s="55">
+        <f>IF(H64&lt;=B7,I63*(1+E15)+B11*12,MAX(0,I63*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J64" s="55">
+        <f>IF(H64&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="G65" s="52" t="n">
+        <v>30</v>
+      </c>
+      <c r="H65" s="52">
+        <f>B6+G65</f>
+        <v/>
+      </c>
+      <c r="I65" s="53">
+        <f>IF(H65&lt;=B7,I64*(1+E15)+B11*12,MAX(0,I64*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J65" s="53">
+        <f>IF(H65&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="G66" s="54" t="n">
+        <v>31</v>
+      </c>
+      <c r="H66" s="54">
+        <f>B6+G66</f>
+        <v/>
+      </c>
+      <c r="I66" s="55">
+        <f>IF(H66&lt;=B7,I65*(1+E15)+B11*12,MAX(0,I65*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J66" s="55">
+        <f>IF(H66&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="G67" s="52" t="n">
+        <v>32</v>
+      </c>
+      <c r="H67" s="52">
+        <f>B6+G67</f>
+        <v/>
+      </c>
+      <c r="I67" s="53">
+        <f>IF(H67&lt;=B7,I66*(1+E15)+B11*12,MAX(0,I66*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J67" s="53">
+        <f>IF(H67&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="G68" s="54" t="n">
+        <v>33</v>
+      </c>
+      <c r="H68" s="54">
+        <f>B6+G68</f>
+        <v/>
+      </c>
+      <c r="I68" s="55">
+        <f>IF(H68&lt;=B7,I67*(1+E15)+B11*12,MAX(0,I67*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J68" s="55">
+        <f>IF(H68&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="G69" s="52" t="n">
+        <v>34</v>
+      </c>
+      <c r="H69" s="52">
+        <f>B6+G69</f>
+        <v/>
+      </c>
+      <c r="I69" s="53">
+        <f>IF(H69&lt;=B7,I68*(1+E15)+B11*12,MAX(0,I68*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J69" s="53">
+        <f>IF(H69&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="G70" s="54" t="n">
+        <v>35</v>
+      </c>
+      <c r="H70" s="54">
+        <f>B6+G70</f>
+        <v/>
+      </c>
+      <c r="I70" s="55">
+        <f>IF(H70&lt;=B7,I69*(1+E15)+B11*12,MAX(0,I69*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J70" s="55">
+        <f>IF(H70&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="G71" s="52" t="n">
+        <v>36</v>
+      </c>
+      <c r="H71" s="52">
+        <f>B6+G71</f>
+        <v/>
+      </c>
+      <c r="I71" s="53">
+        <f>IF(H71&lt;=B7,I70*(1+E15)+B11*12,MAX(0,I70*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J71" s="53">
+        <f>IF(H71&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="G72" s="54" t="n">
+        <v>37</v>
+      </c>
+      <c r="H72" s="54">
+        <f>B6+G72</f>
+        <v/>
+      </c>
+      <c r="I72" s="55">
+        <f>IF(H72&lt;=B7,I71*(1+E15)+B11*12,MAX(0,I71*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J72" s="55">
+        <f>IF(H72&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="G73" s="52" t="n">
+        <v>38</v>
+      </c>
+      <c r="H73" s="52">
+        <f>B6+G73</f>
+        <v/>
+      </c>
+      <c r="I73" s="53">
+        <f>IF(H73&lt;=B7,I72*(1+E15)+B11*12,MAX(0,I72*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J73" s="53">
+        <f>IF(H73&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="G74" s="54" t="n">
+        <v>39</v>
+      </c>
+      <c r="H74" s="54">
+        <f>B6+G74</f>
+        <v/>
+      </c>
+      <c r="I74" s="55">
+        <f>IF(H74&lt;=B7,I73*(1+E15)+B11*12,MAX(0,I73*(1+E16)-B18))</f>
+        <v/>
+      </c>
+      <c r="J74" s="55">
+        <f>IF(H74&lt;B7,NA(),B21)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="G33:J33"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TABELA PERIÓDICA DOS INVESTIMENTOS — RETORNO ANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Índice / Classe</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Acumulado</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="56" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="B4" s="57" t="n"/>
+      <c r="C4" s="57" t="n"/>
+      <c r="D4" s="57" t="n"/>
+      <c r="E4" s="57" t="n"/>
+      <c r="F4" s="57" t="n"/>
+      <c r="G4" s="57" t="n"/>
+      <c r="H4" s="57" t="n"/>
+      <c r="I4" s="57" t="n"/>
+      <c r="J4" s="58">
+        <f>IFERROR(PRODUCT(IF(ISNUMBER(B4:I4),1+B4:I4,1))-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="59" t="inlineStr">
+        <is>
+          <t>Euro Stoxx 50</t>
+        </is>
+      </c>
+      <c r="B5" s="57" t="n"/>
+      <c r="C5" s="57" t="n"/>
+      <c r="D5" s="57" t="n"/>
+      <c r="E5" s="57" t="n"/>
+      <c r="F5" s="57" t="n"/>
+      <c r="G5" s="57" t="n"/>
+      <c r="H5" s="57" t="n"/>
+      <c r="I5" s="57" t="n"/>
+      <c r="J5" s="58">
+        <f>IFERROR(PRODUCT(IF(ISNUMBER(B5:I5),1+B5:I5,1))-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="56" t="inlineStr">
+        <is>
+          <t>Ibovespa</t>
+        </is>
+      </c>
+      <c r="B6" s="57" t="n"/>
+      <c r="C6" s="57" t="n"/>
+      <c r="D6" s="57" t="n"/>
+      <c r="E6" s="57" t="n"/>
+      <c r="F6" s="57" t="n"/>
+      <c r="G6" s="57" t="n"/>
+      <c r="H6" s="57" t="n"/>
+      <c r="I6" s="57" t="n"/>
+      <c r="J6" s="58">
+        <f>IFERROR(PRODUCT(IF(ISNUMBER(B6:I6),1+B6:I6,1))-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="59" t="inlineStr">
+        <is>
+          <t>IFIX</t>
+        </is>
+      </c>
+      <c r="B7" s="57" t="n"/>
+      <c r="C7" s="57" t="n"/>
+      <c r="D7" s="57" t="n"/>
+      <c r="E7" s="57" t="n"/>
+      <c r="F7" s="57" t="n"/>
+      <c r="G7" s="57" t="n"/>
+      <c r="H7" s="57" t="n"/>
+      <c r="I7" s="57" t="n"/>
+      <c r="J7" s="58">
+        <f>IFERROR(PRODUCT(IF(ISNUMBER(B7:I7),1+B7:I7,1))-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="56" t="inlineStr">
+        <is>
+          <t>IMA-B</t>
+        </is>
+      </c>
+      <c r="B8" s="57" t="n"/>
+      <c r="C8" s="57" t="n"/>
+      <c r="D8" s="57" t="n"/>
+      <c r="E8" s="57" t="n"/>
+      <c r="F8" s="57" t="n"/>
+      <c r="G8" s="57" t="n"/>
+      <c r="H8" s="57" t="n"/>
+      <c r="I8" s="57" t="n"/>
+      <c r="J8" s="58">
+        <f>IFERROR(PRODUCT(IF(ISNUMBER(B8:I8),1+B8:I8,1))-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="59" t="inlineStr">
+        <is>
+          <t>IRF-M</t>
+        </is>
+      </c>
+      <c r="B9" s="57" t="n"/>
+      <c r="C9" s="57" t="n"/>
+      <c r="D9" s="57" t="n"/>
+      <c r="E9" s="57" t="n"/>
+      <c r="F9" s="57" t="n"/>
+      <c r="G9" s="57" t="n"/>
+      <c r="H9" s="57" t="n"/>
+      <c r="I9" s="57" t="n"/>
+      <c r="J9" s="58">
+        <f>IFERROR(PRODUCT(IF(ISNUMBER(B9:I9),1+B9:I9,1))-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="56" t="inlineStr">
+        <is>
+          <t>IHFA</t>
+        </is>
+      </c>
+      <c r="B10" s="57" t="n"/>
+      <c r="C10" s="57" t="n"/>
+      <c r="D10" s="57" t="n"/>
+      <c r="E10" s="57" t="n"/>
+      <c r="F10" s="57" t="n"/>
+      <c r="G10" s="57" t="n"/>
+      <c r="H10" s="57" t="n"/>
+      <c r="I10" s="57" t="n"/>
+      <c r="J10" s="58">
+        <f>IFERROR(PRODUCT(IF(ISNUMBER(B10:I10),1+B10:I10,1))-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="59" t="inlineStr">
+        <is>
+          <t>CDI</t>
+        </is>
+      </c>
+      <c r="B11" s="57" t="n"/>
+      <c r="C11" s="57" t="n"/>
+      <c r="D11" s="57" t="n"/>
+      <c r="E11" s="57" t="n"/>
+      <c r="F11" s="57" t="n"/>
+      <c r="G11" s="57" t="n"/>
+      <c r="H11" s="57" t="n"/>
+      <c r="I11" s="57" t="n"/>
+      <c r="J11" s="58">
+        <f>IFERROR(PRODUCT(IF(ISNUMBER(B11:I11),1+B11:I11,1))-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="56" t="inlineStr">
+        <is>
+          <t>Dólar</t>
+        </is>
+      </c>
+      <c r="B12" s="57" t="n"/>
+      <c r="C12" s="57" t="n"/>
+      <c r="D12" s="57" t="n"/>
+      <c r="E12" s="57" t="n"/>
+      <c r="F12" s="57" t="n"/>
+      <c r="G12" s="57" t="n"/>
+      <c r="H12" s="57" t="n"/>
+      <c r="I12" s="57" t="n"/>
+      <c r="J12" s="58">
+        <f>IFERROR(PRODUCT(IF(ISNUMBER(B12:I12),1+B12:I12,1))-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="59" t="inlineStr">
+        <is>
+          <t>Inflação</t>
+        </is>
+      </c>
+      <c r="B13" s="57" t="n"/>
+      <c r="C13" s="57" t="n"/>
+      <c r="D13" s="57" t="n"/>
+      <c r="E13" s="57" t="n"/>
+      <c r="F13" s="57" t="n"/>
+      <c r="G13" s="57" t="n"/>
+      <c r="H13" s="57" t="n"/>
+      <c r="I13" s="57" t="n"/>
+      <c r="J13" s="58">
+        <f>IFERROR(PRODUCT(IF(ISNUMBER(B13:I13),1+B13:I13,1))-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="60" t="inlineStr">
+        <is>
+          <t>Preencha os retornos anuais (em %) de cada índice/classe. A coluna Acumulado é calculada automaticamente; a cor destaca os melhores (verde) e piores (vermelho) de cada ano.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A16:J16"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B4:B13">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:C13">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4:D13">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E4:E13">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F4:F13">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:G13">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4:H13">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I4:I13">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="42" t="inlineStr">
+      <c r="A1" s="61" t="inlineStr">
         <is>
           <t>COMO USAR ESTA PLANILHA</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="43" t="inlineStr"/>
+      <c r="A2" s="62" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="44" t="inlineStr">
+      <c r="A3" s="63" t="inlineStr">
         <is>
           <t>1. Aba 'Clientes': cadastre cada cliente uma única vez — Penumper, Nome e CPF. O Penumper é a chave que liga tudo; pode ter letras (ex.: 1297217A), por isso a coluna é formatada como texto.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="43" t="inlineStr">
+      <c r="A4" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve">     Penumper ou CPF repetidos ficam destacados em vermelho.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="43" t="inlineStr"/>
+      <c r="A5" s="62" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="A6" s="63" t="inlineStr">
         <is>
           <t>2. Aba 'Aplicacoes': cole aqui a posição vinda do sistema — Penumper, Mês, Produto, Subproduto, Vencimento, Saldo Ponta e Idade.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="43" t="inlineStr">
+      <c r="A7" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve">     As colunas Nome e CPF se preenchem sozinhas por PROCV usando o Penumper. Se aparecer 'NÃO CADASTRADO', falta cadastrar o cliente na aba 'Clientes'.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="43" t="inlineStr">
+      <c r="A8" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve">     Cada linha é um investimento (um produto/subproduto com saldo).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="43" t="inlineStr"/>
+      <c r="A9" s="62" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="44" t="inlineStr">
+      <c r="A10" s="63" t="inlineStr">
         <is>
           <t>3. Aba 'Carteira do Cliente': escolha o cliente no menu suspenso. A planilha mostra o patrimônio total, a alocação por classe (com gráfico) e a lista das aplicações daquele cliente.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="A11" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve">     A linha 'Não classificado' indica saldo cujo Produto não casou com nenhum filtro — ajuste os filtros da coluna B se isso acontecer.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="43" t="inlineStr"/>
+      <c r="A12" s="62" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="44" t="inlineStr">
+      <c r="A13" s="63" t="inlineStr">
         <is>
           <t>4. Classes: na aba 'Carteira do Cliente' a coluna 'Filtro (contém)' define como cada classe é somada. Ex.: o filtro FUNDOS soma todo Produto que contenha 'FUNDOS'. Edite rótulos e filtros à vontade.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="43" t="inlineStr"/>
+      <c r="A14" s="62" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="44" t="inlineStr">
+      <c r="A15" s="63" t="inlineStr">
         <is>
-          <t>5. Aba 'Carteira Sugerida': à esquerda aparece a carteira atual por classe; à direita você monta manualmente a carteira recomendada (escolha a Classe, descreva o investimento e informe o valor).</t>
+          <t>5. Aba 'Carteira Sugerida' (proposta): monte a carteira recomendada — Classe, Ativo sugerido, Carência (dias), Liquidez (dias) e Valor. O banner 'Patrimônio Proposto' soma sozinho e os dois gráficos (composição por classe e distribuição de liquidez) se atualizam.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="43" t="inlineStr">
+      <c r="A16" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">     O comparativo no fim mostra, classe a classe, o % atual x o % sugerido e quanto Aumentar ou Reduzir para chegar à carteira ideal.</t>
+          <t xml:space="preserve">     Logo abaixo há campos livres para você descrever as Otimizações Realizadas e o Racional por movimentação (objetivo, justificativa).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="43" t="inlineStr"/>
+      <c r="A17" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     O Comparativo no fim mostra, classe a classe, o % atual x o % sugerido e quanto Aumentar ou Reduzir.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="43" t="inlineStr">
+      <c r="A18" s="62" t="inlineStr"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="63" t="inlineStr">
+        <is>
+          <t>6. Aba 'Planejamento': preencha os campos amarelos (idades, patrimônio, aplicação mensal, renda desejada, INSS, premissas de inflação/CDI/IR/taxa real). A planilha calcula sozinha: o patrimônio necessário na aposentadoria nos cenários 'Viver de Renda' (preservando) e 'Consumo com Sucessão', a parcela mensal a aplicar em cada cenário, os objetivos de vida (projetos 1-6 anos) e a Projeção Patrimonial em R$ de hoje (gráfico de área).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="62" t="inlineStr"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="63" t="inlineStr">
+        <is>
+          <t>7. Aba 'Tabela Periódica': preencha os retornos anuais (%) de cada índice/classe nas colunas dos anos. A coluna 'Acumulado' calcula sozinha e a cor destaca, em cada ano, o melhor (verde) e o pior (vermelho) desempenho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="62" t="inlineStr"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="62" t="inlineStr">
         <is>
           <t>Observação: a planilha trabalha com a posição atual (foto). Para acrescentar uma nova posição, basta colar mais linhas na aba 'Aplicacoes' — as fórmulas se estendem automaticamente.</t>
         </is>

</xml_diff>

<commit_message>
Conserta rótulos dos gráficos de rosca
Os rótulos sozinhos com 'X,X%' ficavam soltos perto das fatias sem
indicar de qual produto eram, e os menores se sobrepunham. Agora:

- showCatName + showPercent: cada rótulo vira 'Produto\\nX,X%'
- position = outEnd: rótulos por fora das fatias, com linha de
  chamada para a fatia correspondente
- legend = None: legenda removida (vira redundante já que o nome do
  produto está em cada rótulo)
- charts maiores (Carteira Cliente 11x16, Atual/Proposta 11x14) para
  acomodar os rótulos externos

https://claude.ai/code/session_012B6pvzwHHmCv3nAgYhFWdt
</commit_message>
<xml_diff>
--- a/gestao_carteiras.xlsx
+++ b/gestao_carteiras.xlsx
@@ -455,15 +455,18 @@
           </val>
         </ser>
         <dLbls>
+          <dLblPos val="outEnd"/>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="1"/>
+          <showSerName val="0"/>
           <showPercent val="1"/>
+          <separator val="&#10;"/>
         </dLbls>
         <firstSliceAng val="0"/>
         <holeSize val="10"/>
       </doughnutChart>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -516,15 +519,18 @@
           </val>
         </ser>
         <dLbls>
+          <dLblPos val="outEnd"/>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="1"/>
+          <showSerName val="0"/>
           <showPercent val="1"/>
+          <separator val="&#10;"/>
         </dLbls>
         <firstSliceAng val="0"/>
         <holeSize val="10"/>
       </doughnutChart>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -577,15 +583,18 @@
           </val>
         </ser>
         <dLbls>
+          <dLblPos val="outEnd"/>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="1"/>
+          <showSerName val="0"/>
           <showPercent val="1"/>
+          <separator val="&#10;"/>
         </dLbls>
         <firstSliceAng val="0"/>
         <holeSize val="10"/>
       </doughnutChart>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -601,7 +610,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4680000" cy="3600000"/>
+    <ext cx="5760000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -628,7 +637,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3960000" cy="3240000"/>
+    <ext cx="5040000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -647,10 +656,10 @@
     <from>
       <col>6</col>
       <colOff>0</colOff>
-      <row>23</row>
+      <row>27</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3960000" cy="3240000"/>
+    <ext cx="5040000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>

</xml_diff>

<commit_message>
Corrige corrupção do arquivo nos gráficos de rosca
O openpyxl grava categorias de gráfico sempre como numRef, mesmo
quando os valores são texto (nome de produto). Enquanto os rótulos
só mostravam % isso não dava problema; mas com showCatName=True o
Excel tenta efetivamente usar aqueles textos e detecta a
incompatibilidade de tipo (numérico vs texto) — daí a mensagem
'Encontramos um problema em um conteúdo'.

Helper cat_para_strref() converte cat.numRef para cat.strRef após
set_categories(). Aplicado nos três gráficos de rosca (Carteira do
Cliente, Atual e Proposta na Carteira Sugerida).

https://claude.ai/code/session_012B6pvzwHHmCv3nAgYhFWdt
</commit_message>
<xml_diff>
--- a/gestao_carteiras.xlsx
+++ b/gestao_carteiras.xlsx
@@ -444,9 +444,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Carteira do Cliente'!$A$11:$A$28</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -508,9 +508,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Carteira Sugerida'!$A$8:$A$25</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -572,9 +572,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Carteira Sugerida'!$A$8:$A$25</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>

</xml_diff>

<commit_message>
Troca DoughnutChart por PieChart
O DoughnutChart do OOXML não aceita dLblPos='outEnd' (rótulo por
fora). O Excel marcava os 3 gráficos como inválidos e removia os
desenhos inteiros ('Parte Removida: /xl/drawings/drawing*.xml').

PieChart aceita outEnd, então mantém o layout 'Produto / %' por
fora das fatias com linhas de chamada — visual parecido com a
rosca, sem o furo no meio.

https://claude.ai/code/session_012B6pvzwHHmCv3nAgYhFWdt
</commit_message>
<xml_diff>
--- a/gestao_carteiras.xlsx
+++ b/gestao_carteiras.xlsx
@@ -428,7 +428,7 @@
       </tx>
     </title>
     <plotArea>
-      <doughnutChart>
+      <pieChart>
         <varyColors val="1"/>
         <ser>
           <idx val="0"/>
@@ -464,8 +464,7 @@
           <separator val="&#10;"/>
         </dLbls>
         <firstSliceAng val="0"/>
-        <holeSize val="10"/>
-      </doughnutChart>
+      </pieChart>
     </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -492,7 +491,7 @@
       </tx>
     </title>
     <plotArea>
-      <doughnutChart>
+      <pieChart>
         <varyColors val="1"/>
         <ser>
           <idx val="0"/>
@@ -528,8 +527,7 @@
           <separator val="&#10;"/>
         </dLbls>
         <firstSliceAng val="0"/>
-        <holeSize val="10"/>
-      </doughnutChart>
+      </pieChart>
     </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -556,7 +554,7 @@
       </tx>
     </title>
     <plotArea>
-      <doughnutChart>
+      <pieChart>
         <varyColors val="1"/>
         <ser>
           <idx val="0"/>
@@ -592,8 +590,7 @@
           <separator val="&#10;"/>
         </dLbls>
         <firstSliceAng val="0"/>
-        <holeSize val="10"/>
-      </doughnutChart>
+      </pieChart>
     </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>

</xml_diff>